<commit_message>
Now using v3 data.
</commit_message>
<xml_diff>
--- a/data/BXCC.xlsx
+++ b/data/BXCC.xlsx
@@ -6,9 +6,9 @@
     <workbookView activeTab="0" firstSheet="0" windowHeight="13125" windowWidth="13125" xWindow="0" yWindow="0"/>
   </bookViews>
   <sheets>
-    <sheet name="B" sheetId="4" state="visible" r:id="rId1"/>
-    <sheet name="X" sheetId="5" state="visible" r:id="rId2"/>
-    <sheet name="BX" sheetId="6" state="visible" r:id="rId3"/>
+    <sheet name="B" sheetId="7" state="visible" r:id="rId1"/>
+    <sheet name="X" sheetId="8" state="visible" r:id="rId2"/>
+    <sheet name="BX" sheetId="9" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName localSheetId="2" name="R_">'BX'!$A$235:$BL$259</definedName>
@@ -14000,7 +14000,7 @@
         <v>0</v>
       </c>
       <c r="AK8" s="8">
-        <v>5820.73286270895</v>
+        <v>5820.73286270896</v>
       </c>
       <c r="AL8" s="8">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="AX8" s="8">
-        <v>67354.0211167643</v>
+        <v>67354.0211167639</v>
       </c>
       <c r="AY8" s="8">
         <v>0</v>
@@ -14090,7 +14090,7 @@
         <v>0</v>
       </c>
       <c r="BO8" s="8">
-        <v>3155.64534081532</v>
+        <v>3155.64534081533</v>
       </c>
       <c r="BP8" s="8">
         <v>0</v>
@@ -21665,7 +21665,7 @@
         <v>0</v>
       </c>
       <c r="AJ35" s="8">
-        <v>58054.842038054</v>
+        <v>58054.8420380546</v>
       </c>
       <c r="AK35" s="8">
         <v>0</v>
@@ -21802,7 +21802,7 @@
         <v>0</v>
       </c>
       <c r="CE35" s="8">
-        <v>0.72465121788954</v>
+        <v>0.724651217889545</v>
       </c>
       <c r="CF35" s="8">
         <v>0</v>
@@ -23178,7 +23178,7 @@
         <v>0</v>
       </c>
       <c r="BO40" s="8">
-        <v>4306.09334056137</v>
+        <v>4306.09334056135</v>
       </c>
       <c r="BP40" s="8">
         <v>0</v>
@@ -25062,7 +25062,7 @@
         <v>0</v>
       </c>
       <c r="AK50" s="8">
-        <v>45017.5962724527</v>
+        <v>45017.5962724529</v>
       </c>
       <c r="AL50" s="8">
         <v>0</v>
@@ -25503,7 +25503,7 @@
         <v>0</v>
       </c>
       <c r="AK53" s="8">
-        <v>66251.1826186745</v>
+        <v>66251.1826186753</v>
       </c>
       <c r="AL53" s="8">
         <v>0</v>
@@ -25884,7 +25884,7 @@
         <v>0</v>
       </c>
       <c r="BN55" s="8">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="BO55" s="8">
         <v>0</v>
@@ -26424,7 +26424,7 @@
         <v>0</v>
       </c>
       <c r="AX59" s="8">
-        <v>2511.39823520817</v>
+        <v>2511.39823520821</v>
       </c>
       <c r="AY59" s="8">
         <v>0</v>
@@ -27012,7 +27012,7 @@
         <v>0</v>
       </c>
       <c r="AX63" s="8">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="AY63" s="8">
         <v>0</v>
@@ -27159,7 +27159,7 @@
         <v>0</v>
       </c>
       <c r="AY64" s="8">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="AZ64" s="8">
         <v>0</v>
@@ -28386,7 +28386,7 @@
         <v>0</v>
       </c>
       <c r="AQ73" s="8">
-        <v>10407.5814017372</v>
+        <v>10407.5814017371</v>
       </c>
       <c r="AR73" s="8">
         <v>0</v>
@@ -28576,7 +28576,7 @@
         <v>0</v>
       </c>
       <c r="BH74" s="8">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="BI74" s="8">
         <v>0</v>
@@ -28875,7 +28875,7 @@
         <v>0</v>
       </c>
       <c r="BO76" s="8">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="BP76" s="8">
         <v>0</v>
@@ -29011,7 +29011,7 @@
         <v>0</v>
       </c>
       <c r="BN77" s="8">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="BO77" s="8">
         <v>0</v>
@@ -29147,7 +29147,7 @@
         <v>0</v>
       </c>
       <c r="BM78" s="8">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="BN78" s="8">
         <v>0</v>
@@ -29247,7 +29247,7 @@
         <v>0</v>
       </c>
       <c r="AZ79" s="8">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="BA79" s="8">
         <v>0</v>
@@ -29755,7 +29755,7 @@
         <v>0</v>
       </c>
       <c r="AJ83" s="8">
-        <v>22059.3433863931</v>
+        <v>22059.3433863928</v>
       </c>
       <c r="AK83" s="8">
         <v>0</v>
@@ -29797,7 +29797,7 @@
         <v>0</v>
       </c>
       <c r="AX83" s="8">
-        <v>3204496.14876622</v>
+        <v>3204496.14876626</v>
       </c>
       <c r="AY83" s="8">
         <v>0</v>
@@ -29897,7 +29897,7 @@
         <v>0</v>
       </c>
       <c r="AK84" s="8">
-        <v>3090735.74001444</v>
+        <v>3090735.74001448</v>
       </c>
       <c r="AL84" s="8">
         <v>0</v>
@@ -30153,7 +30153,7 @@
         <v>0</v>
       </c>
       <c r="BX85" s="8">
-        <v>21683.7905613496</v>
+        <v>21683.7905613501</v>
       </c>
       <c r="BY85" s="8">
         <v>0</v>
@@ -30214,7 +30214,7 @@
         <v>0</v>
       </c>
       <c r="AX86" s="8">
-        <v>5048.75518763039</v>
+        <v>5048.75518763036</v>
       </c>
       <c r="AY86" s="8">
         <v>0</v>
@@ -30362,7 +30362,7 @@
         <v>0</v>
       </c>
       <c r="BA87" s="8">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="BB87" s="8">
         <v>0</v>
@@ -30631,7 +30631,7 @@
         <v>0</v>
       </c>
       <c r="AX89" s="8">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="AY89" s="8">
         <v>0</v>
@@ -30782,7 +30782,7 @@
         <v>0</v>
       </c>
       <c r="BB90" s="8">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="BC90" s="8">
         <v>0</v>
@@ -31048,7 +31048,7 @@
         <v>0</v>
       </c>
       <c r="AX92" s="8">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="AY92" s="8">
         <v>0</v>
@@ -31202,7 +31202,7 @@
         <v>0</v>
       </c>
       <c r="BC93" s="8">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="BD93" s="8">
         <v>0</v>
@@ -31733,7 +31733,7 @@
         <v>0</v>
       </c>
       <c r="AJ98" s="7">
-        <v>45017.5962724527</v>
+        <v>45017.5962724529</v>
       </c>
       <c r="AK98" s="7">
         <v>0</v>
@@ -32561,7 +32561,7 @@
         <v>0</v>
       </c>
       <c r="AJ101" s="7">
-        <v>66251.1826186745</v>
+        <v>66251.1826186753</v>
       </c>
       <c r="AK101" s="7">
         <v>0</v>
@@ -33143,7 +33143,7 @@
         <v>0</v>
       </c>
       <c r="AT103" s="7">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="AU103" s="7">
         <v>0</v>
@@ -33389,13 +33389,13 @@
         <v>0</v>
       </c>
       <c r="AJ104" s="7">
-        <v>5820.73286270895</v>
+        <v>5820.73286270896</v>
       </c>
       <c r="AK104" s="7">
         <v>0</v>
       </c>
       <c r="AL104" s="7">
-        <v>67354.0211167643</v>
+        <v>67354.0211167639</v>
       </c>
       <c r="AM104" s="7">
         <v>0</v>
@@ -33422,7 +33422,7 @@
         <v>0</v>
       </c>
       <c r="AU104" s="7">
-        <v>3155.64534081532</v>
+        <v>3155.64534081533</v>
       </c>
       <c r="AV104" s="7">
         <v>0</v>
@@ -34223,7 +34223,7 @@
         <v>0</v>
       </c>
       <c r="AL107" s="7">
-        <v>2511.39823520817</v>
+        <v>2511.39823520821</v>
       </c>
       <c r="AM107" s="7">
         <v>0</v>
@@ -35327,7 +35327,7 @@
         <v>0</v>
       </c>
       <c r="AL111" s="7">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="AM111" s="7">
         <v>0</v>
@@ -35606,7 +35606,7 @@
         <v>0</v>
       </c>
       <c r="AM112" s="7">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="AN112" s="7">
         <v>0</v>
@@ -38084,7 +38084,7 @@
         <v>0</v>
       </c>
       <c r="AK121" s="7">
-        <v>10407.5814017372</v>
+        <v>10407.5814017371</v>
       </c>
       <c r="AL121" s="7">
         <v>0</v>
@@ -38381,7 +38381,7 @@
         <v>0</v>
       </c>
       <c r="AR122" s="7">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="AS122" s="7">
         <v>0</v>
@@ -38942,7 +38942,7 @@
         <v>0</v>
       </c>
       <c r="AU124" s="7">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="AV124" s="7">
         <v>0</v>
@@ -39215,7 +39215,7 @@
         <v>0</v>
       </c>
       <c r="AT125" s="7">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="AU125" s="7">
         <v>0</v>
@@ -39488,7 +39488,7 @@
         <v>0</v>
       </c>
       <c r="AS126" s="7">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="AT126" s="7">
         <v>0</v>
@@ -39749,7 +39749,7 @@
         <v>0</v>
       </c>
       <c r="AN127" s="7">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="AO127" s="7">
         <v>0</v>
@@ -40838,7 +40838,7 @@
         </is>
       </c>
       <c r="AI131" s="7">
-        <v>80114.185424447</v>
+        <v>80114.1854244474</v>
       </c>
       <c r="AJ131" s="7">
         <v>0</v>
@@ -40847,7 +40847,7 @@
         <v>0</v>
       </c>
       <c r="AL131" s="7">
-        <v>3204496.14876622</v>
+        <v>3204496.14876626</v>
       </c>
       <c r="AM131" s="7">
         <v>0</v>
@@ -41117,7 +41117,7 @@
         <v>0</v>
       </c>
       <c r="AJ132" s="7">
-        <v>3090735.74001444</v>
+        <v>3090735.74001448</v>
       </c>
       <c r="AK132" s="7">
         <v>0</v>
@@ -41429,7 +41429,7 @@
         <v>0</v>
       </c>
       <c r="AV133" s="7">
-        <v>21683.7905613496</v>
+        <v>21683.7905613501</v>
       </c>
       <c r="AW133" s="7">
         <v>0</v>
@@ -41675,7 +41675,7 @@
         <v>0</v>
       </c>
       <c r="AL134" s="7">
-        <v>5048.75518763039</v>
+        <v>5048.75518763036</v>
       </c>
       <c r="AM134" s="7">
         <v>0</v>
@@ -41960,7 +41960,7 @@
         <v>0</v>
       </c>
       <c r="AO135" s="7">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="AP135" s="7">
         <v>0</v>
@@ -42254,7 +42254,7 @@
         <v>0</v>
       </c>
       <c r="AU136" s="7">
-        <v>4306.09334056137</v>
+        <v>4306.09334056135</v>
       </c>
       <c r="AV136" s="7">
         <v>0</v>
@@ -42503,7 +42503,7 @@
         <v>0</v>
       </c>
       <c r="AL137" s="7">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="AM137" s="7">
         <v>0</v>
@@ -42791,7 +42791,7 @@
         <v>0</v>
       </c>
       <c r="AP138" s="7">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="AQ138" s="7">
         <v>0</v>
@@ -43331,7 +43331,7 @@
         <v>0</v>
       </c>
       <c r="AL140" s="7">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="AM140" s="7">
         <v>0</v>
@@ -43622,7 +43622,7 @@
         <v>0</v>
       </c>
       <c r="AQ141" s="7">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="AR141" s="7">
         <v>0</v>
@@ -44065,7 +44065,7 @@
         <v>0</v>
       </c>
       <c r="K146" s="7">
-        <v>37142.634115362</v>
+        <v>37142.6341153622</v>
       </c>
       <c r="L146" s="7">
         <v>0</v>
@@ -44104,7 +44104,7 @@
         <v>0</v>
       </c>
       <c r="X146" s="7">
-        <v>16030.3175923004</v>
+        <v>16030.3175923003</v>
       </c>
       <c r="Y146" s="7">
         <v>0</v>
@@ -44159,7 +44159,7 @@
         <v>0</v>
       </c>
       <c r="J147" s="7">
-        <v>5194.92773027326</v>
+        <v>5194.92773027576</v>
       </c>
       <c r="K147" s="7">
         <v>0</v>
@@ -44195,7 +44195,7 @@
         <v>0</v>
       </c>
       <c r="V147" s="7">
-        <v>3202004.51890557</v>
+        <v>3202004.5189056</v>
       </c>
       <c r="W147" s="7">
         <v>0</v>
@@ -44253,7 +44253,7 @@
         <v>0</v>
       </c>
       <c r="I148" s="7">
-        <v>3162.49928465372</v>
+        <v>3162.49928465367</v>
       </c>
       <c r="J148" s="7">
         <v>0</v>
@@ -44298,7 +44298,7 @@
         <v>0</v>
       </c>
       <c r="X148" s="7">
-        <v>5653.47296904925</v>
+        <v>5653.47296904921</v>
       </c>
       <c r="Y148" s="7">
         <v>0</v>
@@ -44368,7 +44368,7 @@
         <v>0</v>
       </c>
       <c r="O149" s="7">
-        <v>813415.740060376</v>
+        <v>813415.740060384</v>
       </c>
       <c r="P149" s="7">
         <v>0</v>
@@ -44456,7 +44456,7 @@
         <v>0</v>
       </c>
       <c r="L150" s="7">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="M150" s="7">
         <v>0</v>
@@ -44577,7 +44577,7 @@
         <v>0</v>
       </c>
       <c r="T151" s="7">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="U151" s="7">
         <v>0</v>
@@ -44689,7 +44689,7 @@
         <v>0</v>
       </c>
       <c r="Y152" s="7">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="Z152" s="7">
         <v>0</v>
@@ -44795,7 +44795,7 @@
         <v>0</v>
       </c>
       <c r="AB153" s="7">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="AC153" s="7">
         <v>0</v>
@@ -44898,7 +44898,7 @@
         <v>0</v>
       </c>
       <c r="AD154" s="7">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="AE154" s="7">
         <v>0</v>
@@ -44953,7 +44953,7 @@
         <v>0</v>
       </c>
       <c r="P155" s="7">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="Q155" s="7">
         <v>0</v>
@@ -45020,7 +45020,7 @@
         <v>0</v>
       </c>
       <c r="F156" s="7">
-        <v>60946.5548992506</v>
+        <v>60946.5548992509</v>
       </c>
       <c r="G156" s="7">
         <v>0</v>
@@ -45111,7 +45111,7 @@
         <v>0</v>
       </c>
       <c r="D157" s="7">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="E157" s="7">
         <v>0</v>
@@ -45129,7 +45129,7 @@
         <v>0</v>
       </c>
       <c r="J157" s="7">
-        <v>0.000000000000101464011453041</v>
+        <v>0</v>
       </c>
       <c r="K157" s="7">
         <v>0</v>
@@ -45153,7 +45153,7 @@
         <v>0</v>
       </c>
       <c r="R157" s="7">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="S157" s="7">
         <v>0</v>
@@ -45220,13 +45220,13 @@
         <v>27606.4545189183</v>
       </c>
       <c r="H158" s="7">
-        <v>60240.4197442838</v>
+        <v>60240.4197442839</v>
       </c>
       <c r="I158" s="7">
         <v>0</v>
       </c>
       <c r="J158" s="7">
-        <v>6738.87888542647</v>
+        <v>6738.87888542642</v>
       </c>
       <c r="K158" s="7">
         <v>0</v>
@@ -45277,7 +45277,7 @@
         <v>0</v>
       </c>
       <c r="AA158" s="7">
-        <v>4306.09334056136</v>
+        <v>4306.09334056135</v>
       </c>
       <c r="AB158" s="7">
         <v>0</v>
@@ -45317,7 +45317,7 @@
         <v>0</v>
       </c>
       <c r="H159" s="7">
-        <v>23202.8958695482</v>
+        <v>23202.8958695483</v>
       </c>
       <c r="I159" s="7">
         <v>0</v>
@@ -45664,7 +45664,7 @@
         <v>0</v>
       </c>
       <c r="F165" s="2">
-        <v>40734.7303283633</v>
+        <v>40734.7303283613</v>
       </c>
       <c r="G165" s="2">
         <v>0</v>
@@ -45764,7 +45764,7 @@
         <v>0</v>
       </c>
       <c r="G166" s="2">
-        <v>872.216637594378</v>
+        <v>872.216637594377</v>
       </c>
       <c r="H166" s="2">
         <v>0</v>
@@ -45864,7 +45864,7 @@
         <v>0</v>
       </c>
       <c r="H167" s="2">
-        <v>36781.3290129294</v>
+        <v>36781.3290129292</v>
       </c>
       <c r="I167" s="2">
         <v>0</v>
@@ -46206,7 +46206,7 @@
         <v>0</v>
       </c>
       <c r="Y170" s="2">
-        <v>24.966118677908</v>
+        <v>24.9661186779879</v>
       </c>
       <c r="Z170" s="2">
         <v>0</v>
@@ -46234,7 +46234,7 @@
         </is>
       </c>
       <c r="B171" s="2">
-        <v>45017.5962724527</v>
+        <v>45017.5962724529</v>
       </c>
       <c r="C171" s="2">
         <v>0</v>
@@ -46334,7 +46334,7 @@
         <v>0</v>
       </c>
       <c r="C172" s="2">
-        <v>66251.1826186745</v>
+        <v>66251.1826186753</v>
       </c>
       <c r="D172" s="2">
         <v>0</v>
@@ -46437,7 +46437,7 @@
         <v>0</v>
       </c>
       <c r="E173" s="2">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="F173" s="2">
         <v>0</v>
@@ -46558,7 +46558,7 @@
         <v>0</v>
       </c>
       <c r="M174" s="2">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="N174" s="2">
         <v>0</v>
@@ -46673,7 +46673,7 @@
         <v>0</v>
       </c>
       <c r="S175" s="2">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="T175" s="2">
         <v>0</v>
@@ -46764,7 +46764,7 @@
         <v>0</v>
       </c>
       <c r="Q176" s="2">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="R176" s="2">
         <v>0</v>
@@ -46873,7 +46873,7 @@
         <v>0</v>
       </c>
       <c r="U177" s="2">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="V177" s="2">
         <v>0</v>
@@ -46976,7 +46976,7 @@
         <v>0</v>
       </c>
       <c r="W178" s="2">
-        <v>3090735.74001444</v>
+        <v>3090735.74001448</v>
       </c>
       <c r="X178" s="2">
         <v>0</v>
@@ -47082,7 +47082,7 @@
         <v>0</v>
       </c>
       <c r="Z179" s="2">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="AA179" s="2">
         <v>0</v>
@@ -47188,7 +47188,7 @@
         <v>0</v>
       </c>
       <c r="AC180" s="2">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="AD180" s="2">
         <v>0</v>
@@ -47291,7 +47291,7 @@
         <v>0</v>
       </c>
       <c r="AE181" s="2">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
     </row>
     <row r="182">
@@ -47316,7 +47316,7 @@
         <v>0</v>
       </c>
       <c r="G182" s="2">
-        <v>633.592333294874</v>
+        <v>633.592333294875</v>
       </c>
       <c r="H182" s="2">
         <v>0</v>
@@ -47361,7 +47361,7 @@
         <v>0</v>
       </c>
       <c r="V182" s="2">
-        <v>82605.8152851038</v>
+        <v>82605.8152850982</v>
       </c>
       <c r="W182" s="2">
         <v>0</v>
@@ -47404,7 +47404,7 @@
         <v>0</v>
       </c>
       <c r="D183" s="2">
-        <v>633.062840553138</v>
+        <v>633.062840553139</v>
       </c>
       <c r="E183" s="2">
         <v>0</v>
@@ -51535,7 +51535,7 @@
         <v>0</v>
       </c>
       <c r="BU21" s="8">
-        <v>5820.73286270895</v>
+        <v>5820.73286270896</v>
       </c>
       <c r="BV21" s="8">
         <v>0</v>
@@ -51568,7 +51568,7 @@
         <v>0</v>
       </c>
       <c r="CF21" s="8">
-        <v>67354.0211167643</v>
+        <v>67354.0211167639</v>
       </c>
       <c r="CG21" s="8">
         <v>0</v>
@@ -51598,7 +51598,7 @@
         <v>0</v>
       </c>
       <c r="CP21" s="8">
-        <v>3155.64534081532</v>
+        <v>3155.64534081533</v>
       </c>
       <c r="CQ21" s="8">
         <v>0</v>
@@ -56770,7 +56770,7 @@
         <v>0</v>
       </c>
       <c r="BT48" s="8">
-        <v>58054.842038054</v>
+        <v>58054.8420380546</v>
       </c>
       <c r="BU48" s="8">
         <v>0</v>
@@ -56862,7 +56862,7 @@
         <v>0</v>
       </c>
       <c r="CZ48" s="8">
-        <v>0.72465121788954</v>
+        <v>0.724651217889545</v>
       </c>
       <c r="DA48" s="8">
         <v>0</v>
@@ -58388,7 +58388,7 @@
         <v>0</v>
       </c>
       <c r="CP56" s="8">
-        <v>4306.09334056137</v>
+        <v>4306.09334056135</v>
       </c>
       <c r="CQ56" s="8">
         <v>0</v>
@@ -60368,7 +60368,7 @@
         <v>0</v>
       </c>
       <c r="BU70" s="8">
-        <v>45017.5962724527</v>
+        <v>45017.5962724529</v>
       </c>
       <c r="BV70" s="8">
         <v>0</v>
@@ -61286,7 +61286,7 @@
         <v>0</v>
       </c>
       <c r="BU79" s="8">
-        <v>66251.1826186745</v>
+        <v>66251.1826186753</v>
       </c>
       <c r="BV79" s="8">
         <v>0</v>
@@ -62033,7 +62033,7 @@
         <v>0</v>
       </c>
       <c r="CO86" s="8">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="CP86" s="8">
         <v>0</v>
@@ -62382,7 +62382,7 @@
         <v>0</v>
       </c>
       <c r="CF90" s="8">
-        <v>2511.39823520817</v>
+        <v>2511.39823520821</v>
       </c>
       <c r="CG90" s="8">
         <v>0</v>
@@ -62758,7 +62758,7 @@
         <v>0</v>
       </c>
       <c r="CF94" s="8">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="CG94" s="8">
         <v>0</v>
@@ -62855,7 +62855,7 @@
         <v>0</v>
       </c>
       <c r="CG95" s="8">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="CH95" s="8">
         <v>0</v>
@@ -64147,7 +64147,7 @@
         <v>10583778.8835768</v>
       </c>
       <c r="BY109" s="8">
-        <v>10407.5814017372</v>
+        <v>10407.5814017371</v>
       </c>
       <c r="BZ109" s="8">
         <v>0</v>
@@ -64283,7 +64283,7 @@
         <v>0</v>
       </c>
       <c r="CM110" s="8">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="CN110" s="8">
         <v>0</v>
@@ -64386,7 +64386,7 @@
         <v>0</v>
       </c>
       <c r="CP111" s="8">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="CQ111" s="8">
         <v>0</v>
@@ -64477,7 +64477,7 @@
         <v>0</v>
       </c>
       <c r="CO112" s="8">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="CP112" s="8">
         <v>0</v>
@@ -64568,7 +64568,7 @@
         <v>0</v>
       </c>
       <c r="CN113" s="8">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="CO113" s="8">
         <v>0</v>
@@ -64644,7 +64644,7 @@
         <v>0</v>
       </c>
       <c r="CH114" s="8">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="CI114" s="8">
         <v>0</v>
@@ -64696,7 +64696,7 @@
         <v>0</v>
       </c>
       <c r="BT115" s="8">
-        <v>22059.3433863931</v>
+        <v>22059.3433863928</v>
       </c>
       <c r="BU115" s="8">
         <v>0</v>
@@ -64732,7 +64732,7 @@
         <v>0</v>
       </c>
       <c r="CF115" s="8">
-        <v>3204496.14876622</v>
+        <v>3204496.14876626</v>
       </c>
       <c r="CG115" s="8">
         <v>0</v>
@@ -64793,7 +64793,7 @@
         <v>0</v>
       </c>
       <c r="BU116" s="8">
-        <v>3090735.74001444</v>
+        <v>3090735.74001448</v>
       </c>
       <c r="BV116" s="8">
         <v>0</v>
@@ -64956,7 +64956,7 @@
         <v>0</v>
       </c>
       <c r="CR117" s="8">
-        <v>21683.7905613496</v>
+        <v>21683.7905613501</v>
       </c>
     </row>
     <row r="118">
@@ -65202,7 +65202,7 @@
         <v>0</v>
       </c>
       <c r="CF120" s="8">
-        <v>5048.75518763039</v>
+        <v>5048.75518763036</v>
       </c>
       <c r="CG120" s="8">
         <v>0</v>
@@ -65305,7 +65305,7 @@
         <v>0</v>
       </c>
       <c r="CI121" s="8">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="CJ121" s="8">
         <v>0</v>
@@ -65578,7 +65578,7 @@
         <v>0</v>
       </c>
       <c r="CF124" s="8">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="CG124" s="8">
         <v>0</v>
@@ -65684,7 +65684,7 @@
         <v>0</v>
       </c>
       <c r="CJ125" s="8">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="CK125" s="8">
         <v>0</v>
@@ -66048,7 +66048,7 @@
         <v>0</v>
       </c>
       <c r="CF129" s="8">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="CG129" s="8">
         <v>0</v>
@@ -66157,7 +66157,7 @@
         <v>0</v>
       </c>
       <c r="CK130" s="8">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="CL130" s="8">
         <v>0</v>
@@ -66566,7 +66566,7 @@
         <v>0</v>
       </c>
       <c r="BU137" s="7">
-        <v>45017.5962724527</v>
+        <v>45017.5962724529</v>
       </c>
       <c r="BV137" s="7">
         <v>0</v>
@@ -67511,7 +67511,7 @@
         <v>0</v>
       </c>
       <c r="BU146" s="7">
-        <v>66251.1826186745</v>
+        <v>66251.1826186753</v>
       </c>
       <c r="BV146" s="7">
         <v>0</v>
@@ -68306,7 +68306,7 @@
         <v>0</v>
       </c>
       <c r="CO153" s="7">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="CP153" s="7">
         <v>0</v>
@@ -68456,7 +68456,7 @@
         <v>0</v>
       </c>
       <c r="BU155" s="7">
-        <v>5820.73286270895</v>
+        <v>5820.73286270896</v>
       </c>
       <c r="BV155" s="7">
         <v>0</v>
@@ -68489,7 +68489,7 @@
         <v>2824.88564774492</v>
       </c>
       <c r="CF155" s="7">
-        <v>67354.0211167643</v>
+        <v>67354.0211167639</v>
       </c>
       <c r="CG155" s="7">
         <v>0</v>
@@ -68519,7 +68519,7 @@
         <v>0</v>
       </c>
       <c r="CP155" s="7">
-        <v>3155.64534081532</v>
+        <v>3155.64534081533</v>
       </c>
       <c r="CQ155" s="7">
         <v>0</v>
@@ -68699,7 +68699,7 @@
         <v>0</v>
       </c>
       <c r="CF157" s="7">
-        <v>2511.39823520817</v>
+        <v>2511.39823520821</v>
       </c>
       <c r="CG157" s="7">
         <v>0</v>
@@ -69119,7 +69119,7 @@
         <v>0</v>
       </c>
       <c r="CF161" s="7">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="CG161" s="7">
         <v>0</v>
@@ -69227,7 +69227,7 @@
         <v>0</v>
       </c>
       <c r="CG162" s="7">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="CH162" s="7">
         <v>0</v>
@@ -70673,7 +70673,7 @@
         <v>10583778.8835768</v>
       </c>
       <c r="BY176" s="7">
-        <v>10407.5814017372</v>
+        <v>10407.5814017371</v>
       </c>
       <c r="BZ176" s="7">
         <v>0</v>
@@ -70820,7 +70820,7 @@
         <v>0</v>
       </c>
       <c r="CM177" s="7">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="CN177" s="7">
         <v>0</v>
@@ -70934,7 +70934,7 @@
         <v>0</v>
       </c>
       <c r="CP178" s="7">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="CQ178" s="7">
         <v>0</v>
@@ -71036,7 +71036,7 @@
         <v>0</v>
       </c>
       <c r="CO179" s="7">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="CP179" s="7">
         <v>0</v>
@@ -71138,7 +71138,7 @@
         <v>0</v>
       </c>
       <c r="CN180" s="7">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="CO180" s="7">
         <v>0</v>
@@ -71225,7 +71225,7 @@
         <v>0</v>
       </c>
       <c r="CH181" s="7">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="CI181" s="7">
         <v>0</v>
@@ -71288,7 +71288,7 @@
         <v>0</v>
       </c>
       <c r="BT182" s="7">
-        <v>80114.185424447</v>
+        <v>80114.1854244474</v>
       </c>
       <c r="BU182" s="7">
         <v>0</v>
@@ -71324,7 +71324,7 @@
         <v>0</v>
       </c>
       <c r="CF182" s="7">
-        <v>3204496.14876622</v>
+        <v>3204496.14876626</v>
       </c>
       <c r="CG182" s="7">
         <v>0</v>
@@ -71396,7 +71396,7 @@
         <v>0</v>
       </c>
       <c r="BU183" s="7">
-        <v>3090735.74001444</v>
+        <v>3090735.74001448</v>
       </c>
       <c r="BV183" s="7">
         <v>0</v>
@@ -71570,7 +71570,7 @@
         <v>0</v>
       </c>
       <c r="CR184" s="7">
-        <v>21683.7905613496</v>
+        <v>21683.7905613501</v>
       </c>
       <c r="CU184" s="3" t="inlineStr">
         <is>
@@ -71849,7 +71849,7 @@
         <v>0</v>
       </c>
       <c r="CF187" s="7">
-        <v>5048.75518763039</v>
+        <v>5048.75518763036</v>
       </c>
       <c r="CG187" s="7">
         <v>0</v>
@@ -71963,7 +71963,7 @@
         <v>0</v>
       </c>
       <c r="CI188" s="7">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="CJ188" s="7">
         <v>0</v>
@@ -72194,7 +72194,7 @@
         <v>0</v>
       </c>
       <c r="CP190" s="7">
-        <v>4306.09334056137</v>
+        <v>4306.09334056135</v>
       </c>
       <c r="CQ190" s="7">
         <v>0</v>
@@ -72269,7 +72269,7 @@
         <v>0</v>
       </c>
       <c r="CF191" s="7">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="CG191" s="7">
         <v>0</v>
@@ -72386,7 +72386,7 @@
         <v>0</v>
       </c>
       <c r="CJ192" s="7">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="CK192" s="7">
         <v>0</v>
@@ -72794,7 +72794,7 @@
         <v>0</v>
       </c>
       <c r="CF196" s="7">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="CG196" s="7">
         <v>0</v>
@@ -72914,7 +72914,7 @@
         <v>0</v>
       </c>
       <c r="CK197" s="7">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="CL197" s="7">
         <v>0</v>
@@ -74246,7 +74246,7 @@
         <v>0</v>
       </c>
       <c r="Z207" s="7">
-        <v>37142.634115362</v>
+        <v>37142.6341153622</v>
       </c>
       <c r="AA207" s="7">
         <v>0</v>
@@ -74318,7 +74318,7 @@
         <v>0</v>
       </c>
       <c r="AX207" s="7">
-        <v>16030.3175923004</v>
+        <v>16030.3175923003</v>
       </c>
       <c r="AY207" s="7">
         <v>0</v>
@@ -74439,7 +74439,7 @@
         <v>0</v>
       </c>
       <c r="Y208" s="7">
-        <v>5194.92773027326</v>
+        <v>5194.92773027576</v>
       </c>
       <c r="Z208" s="7">
         <v>0</v>
@@ -74508,7 +74508,7 @@
         <v>0</v>
       </c>
       <c r="AV208" s="7">
-        <v>3202004.51890557</v>
+        <v>3202004.5189056</v>
       </c>
       <c r="AW208" s="7">
         <v>0</v>
@@ -75220,7 +75220,7 @@
         <v>0</v>
       </c>
       <c r="X212" s="7">
-        <v>3162.49928465372</v>
+        <v>3162.49928465367</v>
       </c>
       <c r="Y212" s="7">
         <v>0</v>
@@ -75298,7 +75298,7 @@
         <v>0</v>
       </c>
       <c r="AX212" s="7">
-        <v>5653.47296904925</v>
+        <v>5653.47296904921</v>
       </c>
       <c r="AY212" s="7">
         <v>0</v>
@@ -76643,7 +76643,7 @@
         <v>0</v>
       </c>
       <c r="AO219" s="7">
-        <v>813415.740060376</v>
+        <v>813415.740060384</v>
       </c>
       <c r="AP219" s="7">
         <v>0</v>
@@ -76797,7 +76797,7 @@
         <v>0</v>
       </c>
       <c r="AA220" s="7">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="AB220" s="7">
         <v>0</v>
@@ -77050,7 +77050,7 @@
         <v>0</v>
       </c>
       <c r="AT221" s="7">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="AU221" s="7">
         <v>0</v>
@@ -77267,7 +77267,7 @@
         <v>0</v>
       </c>
       <c r="BA222" s="7">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="BB222" s="7">
         <v>0</v>
@@ -77475,7 +77475,7 @@
         <v>0</v>
       </c>
       <c r="BE223" s="7">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="BF223" s="7">
         <v>0</v>
@@ -77686,7 +77686,7 @@
         <v>0</v>
       </c>
       <c r="BJ224" s="7">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="BK224" s="7">
         <v>0</v>
@@ -78018,7 +78018,7 @@
         <v>0</v>
       </c>
       <c r="AP226" s="7">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="AQ226" s="7">
         <v>0</v>
@@ -78151,7 +78151,7 @@
         <v>0</v>
       </c>
       <c r="U227" s="7">
-        <v>60946.5548992506</v>
+        <v>60946.5548992509</v>
       </c>
       <c r="V227" s="7">
         <v>0</v>
@@ -78338,7 +78338,7 @@
         <v>0</v>
       </c>
       <c r="R228" s="7">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="S228" s="7">
         <v>0</v>
@@ -78359,7 +78359,7 @@
         <v>0</v>
       </c>
       <c r="Y228" s="7">
-        <v>0.000000000000101464011453041</v>
+        <v>0</v>
       </c>
       <c r="Z228" s="7">
         <v>0</v>
@@ -78416,7 +78416,7 @@
         <v>0</v>
       </c>
       <c r="AR228" s="7">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="AS228" s="7">
         <v>0</v>
@@ -78549,13 +78549,13 @@
         <v>27606.4545189183</v>
       </c>
       <c r="W229" s="7">
-        <v>60240.4197442838</v>
+        <v>60240.4197442839</v>
       </c>
       <c r="X229" s="7">
         <v>0</v>
       </c>
       <c r="Y229" s="7">
-        <v>6738.87888542647</v>
+        <v>6738.87888542642</v>
       </c>
       <c r="Z229" s="7">
         <v>0</v>
@@ -78648,7 +78648,7 @@
         <v>0</v>
       </c>
       <c r="BD229" s="7">
-        <v>4306.09334056136</v>
+        <v>4306.09334056135</v>
       </c>
       <c r="BE229" s="7">
         <v>0</v>
@@ -78941,7 +78941,7 @@
         <v>0</v>
       </c>
       <c r="W231" s="7">
-        <v>23202.8958695482</v>
+        <v>23202.8958695483</v>
       </c>
       <c r="X231" s="7">
         <v>0</v>
@@ -79651,7 +79651,7 @@
         <v>0</v>
       </c>
       <c r="U237" s="2">
-        <v>40734.7303283633</v>
+        <v>40734.7303283613</v>
       </c>
       <c r="V237" s="2">
         <v>0</v>
@@ -79850,7 +79850,7 @@
         <v>0</v>
       </c>
       <c r="V238" s="2">
-        <v>872.216637594378</v>
+        <v>872.216637594377</v>
       </c>
       <c r="W238" s="2">
         <v>0</v>
@@ -80049,7 +80049,7 @@
         <v>0</v>
       </c>
       <c r="W239" s="2">
-        <v>36781.3290129294</v>
+        <v>36781.3290129292</v>
       </c>
       <c r="X239" s="2">
         <v>0</v>
@@ -80727,7 +80727,7 @@
         <v>0</v>
       </c>
       <c r="BA242" s="2">
-        <v>24.966118677908</v>
+        <v>24.9661186779879</v>
       </c>
       <c r="BB242" s="2">
         <v>0</v>
@@ -80773,7 +80773,7 @@
         <v>0</v>
       </c>
       <c r="C243" s="2">
-        <v>45017.5962724527</v>
+        <v>45017.5962724529</v>
       </c>
       <c r="D243" s="2">
         <v>0</v>
@@ -81192,7 +81192,7 @@
         <v>0</v>
       </c>
       <c r="L245" s="2">
-        <v>66251.1826186745</v>
+        <v>66251.1826186753</v>
       </c>
       <c r="M245" s="2">
         <v>0</v>
@@ -81605,7 +81605,7 @@
         <v>0</v>
       </c>
       <c r="S247" s="2">
-        <v>290.153801920188</v>
+        <v>290.153801920193</v>
       </c>
       <c r="T247" s="2">
         <v>0</v>
@@ -81828,7 +81828,7 @@
         <v>0</v>
       </c>
       <c r="AB248" s="2">
-        <v>4830.44426252758</v>
+        <v>4830.44426252755</v>
       </c>
       <c r="AC248" s="2">
         <v>0</v>
@@ -82467,7 +82467,7 @@
         <v>0</v>
       </c>
       <c r="AS251" s="2">
-        <v>668.843689185036</v>
+        <v>668.84368918504</v>
       </c>
       <c r="AT251" s="2">
         <v>0</v>
@@ -82657,7 +82657,7 @@
         <v>0</v>
       </c>
       <c r="AQ252" s="2">
-        <v>3749358.38011217</v>
+        <v>3749358.38011219</v>
       </c>
       <c r="AR252" s="2">
         <v>0</v>
@@ -82865,7 +82865,7 @@
         <v>0</v>
       </c>
       <c r="AU253" s="2">
-        <v>184686.529997729</v>
+        <v>184686.529997727</v>
       </c>
       <c r="AV253" s="2">
         <v>0</v>
@@ -83067,7 +83067,7 @@
         <v>0</v>
       </c>
       <c r="AW254" s="2">
-        <v>3090735.74001444</v>
+        <v>3090735.74001448</v>
       </c>
       <c r="AX254" s="2">
         <v>0</v>
@@ -83278,7 +83278,7 @@
         <v>0</v>
       </c>
       <c r="BB255" s="2">
-        <v>5023.78906895248</v>
+        <v>5023.78906895237</v>
       </c>
       <c r="BC255" s="2">
         <v>0</v>
@@ -83486,7 +83486,7 @@
         <v>0</v>
       </c>
       <c r="BF256" s="2">
-        <v>82.0916287907192</v>
+        <v>82.0916287907193</v>
       </c>
       <c r="BG256" s="2">
         <v>0</v>
@@ -83697,7 +83697,7 @@
         <v>0</v>
       </c>
       <c r="BK257" s="2">
-        <v>43.206120416168</v>
+        <v>43.2061204161677</v>
       </c>
       <c r="BL257" s="2">
         <v>0</v>
@@ -83770,7 +83770,7 @@
         <v>0</v>
       </c>
       <c r="V258" s="2">
-        <v>633.592333294874</v>
+        <v>633.592333294875</v>
       </c>
       <c r="W258" s="2">
         <v>0</v>
@@ -83848,7 +83848,7 @@
         <v>0</v>
       </c>
       <c r="AV258" s="2">
-        <v>82605.8152851038</v>
+        <v>82605.8152850982</v>
       </c>
       <c r="AW258" s="2">
         <v>0</v>
@@ -83954,7 +83954,7 @@
         <v>0</v>
       </c>
       <c r="R259" s="2">
-        <v>633.062840553138</v>
+        <v>633.062840553139</v>
       </c>
       <c r="S259" s="2">
         <v>0</v>

</xml_diff>